<commit_message>
Various changes added and bugs fixed
</commit_message>
<xml_diff>
--- a/Assets/Gifts/EuroGifts.xlsx
+++ b/Assets/Gifts/EuroGifts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\konstantinos\source\repos\EuroSearchApp\Assets\Gifts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86967178-88A5-4D8C-830B-800A8438098D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19659A9A-5D10-4DE4-BA7D-DB8828C0E05C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F48EC37B-4F34-4BD7-AAFD-36B68C903084}"/>
+    <workbookView xWindow="780" yWindow="0" windowWidth="14610" windowHeight="15480" xr2:uid="{F48EC37B-4F34-4BD7-AAFD-36B68C903084}"/>
   </bookViews>
   <sheets>
     <sheet name="Φύλλο1" sheetId="1" r:id="rId1"/>
@@ -25,33 +25,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="16">
-  <si>
-    <t>POWERTECH EARPHONES ME ΘΗΚΗ ΦΟΡΤΙΣΗΣ ΜΑΥΡΟ</t>
-  </si>
-  <si>
-    <t>POWERTECH CABLE USB-C TO USB-C</t>
-  </si>
-  <si>
-    <t>USAMS - ΘΗΚΗ ΑΚΟΥΣΤΙΚΩΝ BLUETOOTH</t>
-  </si>
-  <si>
-    <t>KAKUSIGA EPITRAPEZIA ΒΑΣΗ SMARTPHONE</t>
-  </si>
-  <si>
-    <t>INTIME MAGIC WALLET  / MONEY CLIP</t>
-  </si>
-  <si>
-    <t>PHILIPS ΦΟΡΗΤΟΣ ΦΑΚΟΣ</t>
-  </si>
-  <si>
-    <t>ISOTHERMAL WATERPROOF BAG ( 20 RED + 20 BLUE)</t>
-  </si>
-  <si>
-    <t>KSG 1270 SCANNER ΕΝΣΥΡΜΑΤΟ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EUROMEDICA TWO (Δεν συμψηφίζεται με άλλου είδους μορφή έκπτωσης. Το κουπόνι δώρου μπορεί να μεταβιβαστεί) </t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+  <si>
+    <t xml:space="preserve">ΕΙΔΟΣ </t>
   </si>
   <si>
     <t>50% έκπτωση στη συνδρομή . (Το κουπόνι δώρου δεν ανταλλάσσεται με άλλο είδος και δεν συμψηφίζεται με άλλου είδους μορφή έκπτωσης)</t>
@@ -60,16 +36,110 @@
     <t>20% έκπτωση στη συνδρομή. (Το κουπόνι δώρου δεν ανταλλάσσεται με άλλο είδος και δεν συμψηφίζεται με άλλου είδους μορφή έκπτωσης)</t>
   </si>
   <si>
-    <t>20% έκπτωση στην αρχική τιμή στο πρόγραμμα. Δεν συμψηφίζεται με άλλου είδους μορφή έκπτωσης. Το κουπόνι δώρου μπορεί να μεταβιβαστεί</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> EUROPHARMACY IKE</t>
-  </si>
-  <si>
-    <t>ΧΟ TABLET ΠΑΙΔΙΚΟ ΜΠΛΕ</t>
-  </si>
-  <si>
-    <t>ΕΙΔΟΣ</t>
+    <t>F- anazitisi (Η εξαργύρωση του δώρου ισχύει μόνο εάν ολοκληρωθεί η εγκατάσταση / ανανέωση της υπηρεσίας εντός τριμήνου στο Euromedica TWO)</t>
+  </si>
+  <si>
+    <t>10% έκπτωση στη συνδρομή. (Το κουπόνι δώρου δεν ανταλλάσσεται με άλλο είδος και δεν συμψηφίζεται με άλλου είδους μορφή έκπτωσης)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EUROMEDICA TWO (Δεν συνδυάζεται με άλλου είδους μορφή έκπτωσης. Το κουπόνι δώρου μπορεί να μεταβιβαστεί) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">10% EUROMEDICA TWO (Δεν συνδυάζεται με άλλου είδους μορφή έκπτωσης. Το κουπόνι δώρου μπορεί να μεταβιβαστεί) </t>
+  </si>
+  <si>
+    <t>20% έκπτωση στην αρχική τιμή στο πρόγραμμα. Δεν συνδυάζεται με άλλου είδους μορφή έκπτωσης. Το κουπόνι δώρου μπορεί να μεταβιβαστεί</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ΑΚΟΥΣΤΙΚΑ ME ΘΗΚΗ ΦΟΡΤΙΣΗΣ ΜΑΥΡΟ POWERTECH </t>
+  </si>
+  <si>
+    <t>ΚΑΛΩΔΙΟ USB-C TO USB-C POWERTECH</t>
+  </si>
+  <si>
+    <t>ΘΗΚΗ ΑΚΟΥΣΤΙΚΩΝ BLUETOOTH USAMS</t>
+  </si>
+  <si>
+    <t>ΕΠΙΤΡΑΠΕΖΙΑ ΒΑΣΗ SMARTPHONE KAKUSIGA</t>
+  </si>
+  <si>
+    <t>ΠΟΡΤΟΦΟΛΙ MAGIC WALLET / MONEY CLIP</t>
+  </si>
+  <si>
+    <t>ΦΟΡΗΤΟΣ ΦΑΚΟΣ PHILIPS</t>
+  </si>
+  <si>
+    <t>ΙΣΟΘΕΡΜΙΚΗ ΑΔΙΑΒΡΟΧΗ ΤΣΑΝΤΑ ΦΑΓΗΤΟΥ</t>
+  </si>
+  <si>
+    <t>ΕΝΣΥΡΜΑΤΟ QR SCANNER KSG 1270</t>
+  </si>
+  <si>
+    <t>ΚΑΛΩΔΙΟ ΦΟΡΤΙΣΗΣ NG 5Α TYPE C ROCKET</t>
+  </si>
+  <si>
+    <t>ΠΑΚΕΤΟ ΠΑΡΟΧΟΥ της εταιρίας Parochos</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">ΑΚΟΥΣΤΙΚΑ </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="161"/>
+      </rPr>
+      <t>CHORUS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="161"/>
+      </rPr>
+      <t xml:space="preserve"> STEREO WITH MICROPHONE NG </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">ΑΚΟΥΣΤΙΚΑ </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="161"/>
+      </rPr>
+      <t>MAESTRO</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="2"/>
+        <charset val="161"/>
+      </rPr>
+      <t xml:space="preserve"> STEREO WITH MICROPHONE NG </t>
+    </r>
+  </si>
+  <si>
+    <t>ΚΑΛΩΔΙΟ ΦΟΡΤΙΣΗΣ  BLAZE LIGHTNING GOLD WK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ΦΟΡΤΙΣΤΗΣ ΑΥΤΟΚΙΝΗΤΟΥ ΜΑΥΡΟΣ NG </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ΦΟΡΤΙΣΤΗΣ ΑΥΤΟΚΙΝΗΤΟΥ NG WOOT WT61 </t>
   </si>
   <si>
     <t>ΤΕΜΑΧΙΑ</t>
@@ -111,13 +181,6 @@
       <charset val="161"/>
     </font>
     <font>
-      <sz val="14"/>
-      <color rgb="FF00B050"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-      <charset val="161"/>
-    </font>
-    <font>
       <sz val="8"/>
       <color rgb="FF00B050"/>
       <name val="Tahoma"/>
@@ -131,18 +194,33 @@
       <charset val="161"/>
     </font>
     <font>
-      <sz val="8"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Tahoma"/>
       <family val="2"/>
       <charset val="161"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -169,39 +247,33 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Κανονικό 2" xfId="1" xr:uid="{7A51B82B-834E-45E2-8D9D-60EAEBFE6B05}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -513,167 +585,203 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7CB14EA-9DCF-421E-B4E0-E447C4D46EF4}">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr defaultRowHeight="10.5" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="91.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.5" customWidth="1"/>
-    <col min="3" max="3" width="48.6640625" customWidth="1"/>
+    <col min="1" max="1" width="88.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:2" s="1" customFormat="1" ht="18" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="18" x14ac:dyDescent="0.25">
+      <c r="A2" s="6"/>
+      <c r="B2" s="2"/>
+    </row>
+    <row r="3" spans="1:2" ht="18" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="18" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="18" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="18" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="18" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="18" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="18" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B9" s="2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="7"/>
-    </row>
-    <row r="2" spans="1:3" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="11">
+      <c r="B10" s="2">
         <v>30</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+    </row>
+    <row r="11" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" s="2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" s="2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B18" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" s="3" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" s="3" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B20" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" s="3" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="11">
-        <v>50</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="18" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="B21" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" s="3" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="11">
+      <c r="B22" s="4">
         <v>20</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="18" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="11">
+    </row>
+    <row r="23" spans="1:2" s="3" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B23" s="4">
         <v>20</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="18" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+    </row>
+    <row r="24" spans="1:2" s="3" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="11">
-        <v>30</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="18" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="11">
-        <v>30</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="18" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="11">
-        <v>40</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="11">
-        <v>25</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" s="6" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" s="12">
-        <v>2</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" s="6" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" s="12">
-        <v>20</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" s="6" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+      <c r="B24" s="4">
         <v>10</v>
       </c>
-      <c r="B12" s="12">
-        <v>20</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" s="6" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" s="12">
-        <v>20</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" s="10" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" s="13">
-        <v>99</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>12</v>
-      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>